<commit_message>
user can send summarization
</commit_message>
<xml_diff>
--- a/sellingReport.xlsx
+++ b/sellingReport.xlsx
@@ -5,7 +5,7 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Tickets sold by " sheetId="1" r:id="rId1"/>
+    <sheet name="Tickets sold by Langenkamp" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -25,7 +25,7 @@
     <t>Ticket fee</t>
   </si>
   <si>
-    <t>Total Amount in Eur</t>
+    <t>Total</t>
   </si>
   <si>
     <t>Die Gewitterschwimmerin</t>
@@ -143,13 +143,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>12</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>48</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:5">

</xml_diff>